<commit_message>
Add BCH bank credit to agriculture 2017-2026 to the Honduras year-by-year table
Loans outstanding and new loans to all agriculture (BCH, coffee not
separated) with year-on-year changes; Jan-Jul 2026 new loans +84 % on
Jan-Jul 2025. 2025 Bono volume marked as read.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GCSUFXh2mYdWNgg7VCeE1G
</commit_message>
<xml_diff>
--- a/research/honduras/excel/Honduras_YoY_productivity_inputs_finance_fx.xlsx
+++ b/research/honduras/excel/Honduras_YoY_productivity_inputs_finance_fx.xlsx
@@ -20,12 +20,13 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="5">
+  <numFmts count="6">
     <numFmt numFmtId="164" formatCode="#,##0"/>
     <numFmt numFmtId="165" formatCode="#,##0.0"/>
     <numFmt numFmtId="166" formatCode="0.000"/>
     <numFmt numFmtId="167" formatCode="0.00"/>
     <numFmt numFmtId="168" formatCode="+0.0%;-0.0%;0.0%"/>
+    <numFmt numFmtId="169" formatCode="0.0%"/>
   </numFmts>
   <fonts count="8">
     <font>
@@ -116,7 +117,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -142,6 +143,7 @@
     <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -236,7 +238,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Finance: state and bank programmes by year, debt, Bono Cafetalero.</t>
+          <t xml:space="preserve">Finance: state and bank programmes by year, debt, Bono Cafetalero, BCH bank credit to agriculture 2017-2026.</t>
         </is>
       </c>
     </row>
@@ -6635,6 +6637,367 @@
         </is>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Bank credit to agriculture (BCH, all farming: coffee is not separated), millions of lempiras</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Year</t>
+        </is>
+      </c>
+      <c r="B21" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Loans outstanding, December</t>
+        </is>
+      </c>
+      <c r="C21" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">change</t>
+        </is>
+      </c>
+      <c r="D21" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">New loans in the year</t>
+        </is>
+      </c>
+      <c r="E21" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">change</t>
+        </is>
+      </c>
+      <c r="F21" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Share of all new loans</t>
+        </is>
+      </c>
+      <c r="G21" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Loans outstanding in US$ M</t>
+        </is>
+      </c>
+      <c r="H21" s="4" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Source</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22">
+        <v>2017</v>
+      </c>
+      <c r="B22" s="6">
+        <v>20610.3</v>
+      </c>
+      <c r="D22" s="6">
+        <v>10924.8</v>
+      </c>
+      <c r="F22" s="19">
+        <v>0.04678030027293646</v>
+      </c>
+      <c r="G22" s="9">
+        <f>B22/YoY!AF18</f>
+        <v>877.529508507812</v>
+      </c>
+      <c r="H22" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BCH, Prestamos de las Otras Sociedades de Depositos por Actividad (xlsx read, raw/ihcafe_docs5)</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23">
+        <v>2018</v>
+      </c>
+      <c r="B23" s="6">
+        <v>24314.800000000003</v>
+      </c>
+      <c r="C23" s="13">
+        <f>B23/B22-1</f>
+        <v>0.17974022697389191</v>
+      </c>
+      <c r="D23" s="6">
+        <v>16237.0</v>
+      </c>
+      <c r="E23" s="13">
+        <f>D23/D22-1</f>
+        <v>0.4862514645577036</v>
+      </c>
+      <c r="F23" s="19">
+        <v>0.061453298407482634</v>
+      </c>
+      <c r="G23" s="9">
+        <f>B23/YoY!AF19</f>
+        <v>1017.3081259499902</v>
+      </c>
+      <c r="H23" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BCH, Prestamos de las Otras Sociedades de Depositos por Actividad (xlsx read, raw/ihcafe_docs5)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24">
+        <v>2019</v>
+      </c>
+      <c r="B24" s="6">
+        <v>25923.5</v>
+      </c>
+      <c r="C24" s="13">
+        <f>B24/B23-1</f>
+        <v>0.06616135028871284</v>
+      </c>
+      <c r="D24" s="6">
+        <v>15389.3</v>
+      </c>
+      <c r="E24" s="13">
+        <f>D24/D23-1</f>
+        <v>-0.052207920182299694</v>
+      </c>
+      <c r="F24" s="19">
+        <v>0.05743827810199472</v>
+      </c>
+      <c r="G24" s="9">
+        <f>B24/YoY!AF20</f>
+        <v>1057.7726044736592</v>
+      </c>
+      <c r="H24" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BCH, Prestamos de las Otras Sociedades de Depositos por Actividad (xlsx read, raw/ihcafe_docs5)</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25">
+        <v>2020</v>
+      </c>
+      <c r="B25" s="6">
+        <v>23787.4</v>
+      </c>
+      <c r="C25" s="13">
+        <f>B25/B24-1</f>
+        <v>-0.08240013887013709</v>
+      </c>
+      <c r="D25" s="6">
+        <v>14129.4</v>
+      </c>
+      <c r="E25" s="13">
+        <f>D25/D24-1</f>
+        <v>-0.08186857102012435</v>
+      </c>
+      <c r="F25" s="19">
+        <v>0.050463440488469714</v>
+      </c>
+      <c r="G25" s="9">
+        <f>B25/YoY!AF21</f>
+        <v>967.6639383058496</v>
+      </c>
+      <c r="H25" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BCH, Prestamos de las Otras Sociedades de Depositos por Actividad (xlsx read, raw/ihcafe_docs5)</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26">
+        <v>2021</v>
+      </c>
+      <c r="B26" s="6">
+        <v>25569.699999999997</v>
+      </c>
+      <c r="C26" s="13">
+        <f>B26/B25-1</f>
+        <v>0.07492622144496641</v>
+      </c>
+      <c r="D26" s="6">
+        <v>14373.699999999999</v>
+      </c>
+      <c r="E26" s="13">
+        <f>D26/D25-1</f>
+        <v>0.017290189250781962</v>
+      </c>
+      <c r="F26" s="19">
+        <v>0.04722363951584739</v>
+      </c>
+      <c r="G26" s="9">
+        <f>B26/YoY!AF22</f>
+        <v>1064.7271107811914</v>
+      </c>
+      <c r="H26" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BCH, Prestamos de las Otras Sociedades de Depositos por Actividad (xlsx read, raw/ihcafe_docs5)</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27">
+        <v>2022</v>
+      </c>
+      <c r="B27" s="6">
+        <v>27310.5</v>
+      </c>
+      <c r="C27" s="13">
+        <f>B27/B26-1</f>
+        <v>0.06808057974868698</v>
+      </c>
+      <c r="D27" s="6">
+        <v>15012.9</v>
+      </c>
+      <c r="E27" s="13">
+        <f>D27/D26-1</f>
+        <v>0.04447010860112566</v>
+      </c>
+      <c r="F27" s="19">
+        <v>0.03977877627978923</v>
+      </c>
+      <c r="G27" s="9">
+        <f>B27/YoY!AF23</f>
+        <v>1115.3123569556742</v>
+      </c>
+      <c r="H27" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BCH, Prestamos de las Otras Sociedades de Depositos por Actividad (xlsx read, raw/ihcafe_docs5)</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28">
+        <v>2023</v>
+      </c>
+      <c r="B28" s="6">
+        <v>27976.06574996</v>
+      </c>
+      <c r="C28" s="13">
+        <f>B28/B27-1</f>
+        <v>0.02437032459896371</v>
+      </c>
+      <c r="D28" s="6">
+        <v>15346.5</v>
+      </c>
+      <c r="E28" s="13">
+        <f>D28/D27-1</f>
+        <v>0.022220890034570395</v>
+      </c>
+      <c r="F28" s="19">
+        <v>0.03555675109092603</v>
+      </c>
+      <c r="G28" s="9">
+        <f>B28/YoY!AF24</f>
+        <v>1137.1653556893434</v>
+      </c>
+      <c r="H28" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BCH, Prestamos de las Otras Sociedades de Depositos por Actividad (xlsx read, raw/ihcafe_docs5)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29">
+        <v>2024</v>
+      </c>
+      <c r="B29" s="6">
+        <v>30700.613323690002</v>
+      </c>
+      <c r="C29" s="13">
+        <f>B29/B28-1</f>
+        <v>0.09738851767367973</v>
+      </c>
+      <c r="D29" s="6">
+        <v>17038.59566647</v>
+      </c>
+      <c r="E29" s="13">
+        <f>D29/D28-1</f>
+        <v>0.11025938594923912</v>
+      </c>
+      <c r="F29" s="19">
+        <v>0.03404848055528372</v>
+      </c>
+      <c r="G29" s="9">
+        <f>B29/YoY!AF25</f>
+        <v>1238.1779328720474</v>
+      </c>
+      <c r="H29" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BCH, Prestamos de las Otras Sociedades de Depositos por Actividad (xlsx read, raw/ihcafe_docs5)</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30">
+        <v>2025</v>
+      </c>
+      <c r="B30" s="6">
+        <v>31109.74988466</v>
+      </c>
+      <c r="C30" s="13">
+        <f>B30/B29-1</f>
+        <v>0.013326657570527756</v>
+      </c>
+      <c r="D30" s="6">
+        <v>19080.13470844</v>
+      </c>
+      <c r="E30" s="13">
+        <f>D30/D29-1</f>
+        <v>0.11981850393853266</v>
+      </c>
+      <c r="F30" s="19">
+        <v>0.03554160550007587</v>
+      </c>
+      <c r="G30" s="9">
+        <f>B30/YoY!AF26</f>
+        <v>1198.6165014012095</v>
+      </c>
+      <c r="H30" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">BCH, Prestamos de las Otras Sociedades de Depositos por Actividad (xlsx read, raw/ihcafe_docs5)</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026 Jan-Jul</t>
+        </is>
+      </c>
+      <c r="B31" s="6">
+        <v>32548.21990825</v>
+      </c>
+      <c r="C31" s="13">
+        <f>B31/B32-1</f>
+        <v>0.1039674506401238</v>
+      </c>
+      <c r="D31" s="6">
+        <v>19250.33787004</v>
+      </c>
+      <c r="E31" s="13">
+        <f>D31/D32-1</f>
+        <v>0.8361685637942358</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025 Jan-Jul</t>
+        </is>
+      </c>
+      <c r="B32" s="6">
+        <v>29482.95249953</v>
+      </c>
+      <c r="D32" s="6">
+        <v>10483.97094342</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Reading: credit to agriculture grew slower than total credit (its share of new loans fell from 6.1 % in 2018 to 3.4 % in 2024) and fell in 2020 (-8 %). It picked up in 2024-2025 (+11 %, +12 % new loans) and jumped in 2026: new loans Jan-Jul +84 % on Jan-Jul 2025, with average lending rates down 3.8 points (BCH communique, June 2026). Coffee is not separated in BCH data.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Add the August 2017 IHCAFE early-warning bulletin to the Honduras rust list
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01GCSUFXh2mYdWNgg7VCeE1G
</commit_message>
<xml_diff>
--- a/research/honduras/excel/Honduras_YoY_productivity_inputs_finance_fx.xlsx
+++ b/research/honduras/excel/Honduras_YoY_productivity_inputs_finance_fx.xlsx
@@ -5181,7 +5181,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">There is no published yearly series in the files we could reach: IHCAFE early-warning bulletins (monthly, about 1 200 farms) are behind the blocked ihcafe.hn host. Figures below are those printed by USDA or the press.</t>
+          <t xml:space="preserve">There is no published yearly series in the files we could reach: IHCAFE early-warning bulletins (monthly, about 1 200 farms) are no longer served by ihcafe.hn (old links return the home page; checked 25 Sep 2026). Figures below are those printed by USDA or the press.</t>
         </is>
       </c>
     </row>
@@ -5303,29 +5303,26 @@
     </row>
     <row r="8">
       <c r="A8">
-        <v>2020</v>
+        <v>2017</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t xml:space="preserve">end 2020</t>
-        </is>
-      </c>
-      <c r="C8" s="11">
-        <v>20.0</v>
+          <t xml:space="preserve">Aug 2017</t>
+        </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t xml:space="preserve">incidence in 5 departments after hurricanes Eta and Iota</t>
+          <t xml:space="preserve">IHCAFE SAT bulletin No 6: rust on susceptible varieties green alert (low risk); on resistant varieties and berry borer blue alert (minimal risk)</t>
         </is>
       </c>
       <c r="E8" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">✔ USDA report (read)</t>
+          <t xml:space="preserve">✔ document read</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t xml:space="preserve">GAIN 2021</t>
+          <t xml:space="preserve">IHCAFE SAT page (image, read)</t>
         </is>
       </c>
     </row>
@@ -5335,40 +5332,40 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Nov 2020</t>
-        </is>
+          <t xml:space="preserve">end 2020</t>
+        </is>
+      </c>
+      <c r="C9" s="11">
+        <v>20.0</v>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t xml:space="preserve">Eta and Iota: &gt; 4 200 ha of coffee farms hit, &gt; 150 000 qq lost</t>
+          <t xml:space="preserve">incidence in 5 departments after hurricanes Eta and Iota</t>
         </is>
       </c>
       <c r="E9" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">✔ document read</t>
+          <t xml:space="preserve">✔ USDA report (read)</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t xml:space="preserve">La Prensa / EFE 1 Nov 2022 (read)</t>
+          <t xml:space="preserve">GAIN 2021</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10">
-        <v>2022</v>
+        <v>2020</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t xml:space="preserve">2022/23 crop</t>
-        </is>
-      </c>
-      <c r="C10" s="11">
-        <v>20.0</v>
+          <t xml:space="preserve">Nov 2020</t>
+        </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t xml:space="preserve">% of PRODUCTION affected by rust (IHCAFE director)</t>
+          <t xml:space="preserve">Eta and Iota: &gt; 4 200 ha of coffee farms hit, &gt; 150 000 qq lost</t>
         </is>
       </c>
       <c r="E10" s="17" t="inlineStr">
@@ -5388,43 +5385,43 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Apr 2022</t>
+          <t xml:space="preserve">2022/23 crop</t>
         </is>
       </c>
       <c r="C11" s="11">
-        <v>5.42</v>
+        <v>20.0</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t xml:space="preserve">national average incidence (66 % of farms low, 29 % medium, 5 % high)</t>
+          <t xml:space="preserve">% of PRODUCTION affected by rust (IHCAFE director)</t>
         </is>
       </c>
       <c r="E11" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">✔ USDA report (read)</t>
+          <t xml:space="preserve">✔ document read</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t xml:space="preserve">GAIN 2022</t>
+          <t xml:space="preserve">La Prensa / EFE 1 Nov 2022 (read)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12">
-        <v>2023</v>
+        <v>2022</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t xml:space="preserve">May 2023</t>
+          <t xml:space="preserve">Apr 2022</t>
         </is>
       </c>
       <c r="C12" s="11">
-        <v>5.8</v>
+        <v>5.42</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t xml:space="preserve">national average incidence (La Paz 9.7 %, Fco. Morazan 8.2 %)</t>
+          <t xml:space="preserve">national average incidence (66 % of farms low, 29 % medium, 5 % high)</t>
         </is>
       </c>
       <c r="E12" s="17" t="inlineStr">
@@ -5434,35 +5431,35 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t xml:space="preserve">GAIN 2023 (repeated in GAIN 2024)</t>
+          <t xml:space="preserve">GAIN 2022</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13">
-        <v>2024</v>
+        <v>2023</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Mar 2024</t>
+          <t xml:space="preserve">May 2023</t>
         </is>
       </c>
       <c r="C13" s="11">
-        <v>7.38</v>
+        <v>5.8</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t xml:space="preserve">national average incidence</t>
-        </is>
-      </c>
-      <c r="E13" s="18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">⚠ web extract, not read</t>
+          <t xml:space="preserve">national average incidence (La Paz 9.7 %, Fco. Morazan 8.2 %)</t>
+        </is>
+      </c>
+      <c r="E13" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">✔ USDA report (read)</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t xml:space="preserve">web search summary (La Prensa / El Heraldo)</t>
+          <t xml:space="preserve">GAIN 2023 (repeated in GAIN 2024)</t>
         </is>
       </c>
     </row>
@@ -5472,22 +5469,25 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Apr 2024</t>
-        </is>
+          <t xml:space="preserve">Mar 2024</t>
+        </is>
+      </c>
+      <c r="C14" s="11">
+        <v>7.38</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t xml:space="preserve">76 % of sampled farms low, 19 % medium, 5 % high</t>
-        </is>
-      </c>
-      <c r="E14" s="17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">✔ USDA report (read)</t>
+          <t xml:space="preserve">national average incidence</t>
+        </is>
+      </c>
+      <c r="E14" s="18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">⚠ web extract, not read</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t xml:space="preserve">GAIN 2025</t>
+          <t xml:space="preserve">web search summary (La Prensa / El Heraldo)</t>
         </is>
       </c>
     </row>
@@ -5497,40 +5497,37 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t xml:space="preserve">2024</t>
+          <t xml:space="preserve">Apr 2024</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t xml:space="preserve">BCH: exports about 500 000 qq lower than 2023 "due to high rust incidence and labour shortage"</t>
+          <t xml:space="preserve">76 % of sampled farms low, 19 % medium, 5 % high</t>
         </is>
       </c>
       <c r="E15" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">✔ document read</t>
+          <t xml:space="preserve">✔ USDA report (read)</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t xml:space="preserve">El Heraldo 23 Jun 2024 (read)</t>
+          <t xml:space="preserve">GAIN 2025</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16">
-        <v>2025</v>
+        <v>2024</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t xml:space="preserve">Jan-Mar 2025</t>
-        </is>
-      </c>
-      <c r="C16" s="11">
-        <v>5.71</v>
+          <t xml:space="preserve">2024</t>
+        </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t xml:space="preserve">national average (13 of 15 departments hit; Santa Barbara 9.29 %, El Paraiso 7.91 %, Comayagua 7.20 %; worst varieties Obata and Catuai)</t>
+          <t xml:space="preserve">BCH: exports about 500 000 qq lower than 2023 "due to high rust incidence and labour shortage"</t>
         </is>
       </c>
       <c r="E16" s="17" t="inlineStr">
@@ -5540,7 +5537,7 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t xml:space="preserve">El Heraldo 13 May 2025 (read)</t>
+          <t xml:space="preserve">El Heraldo 23 Jun 2024 (read)</t>
         </is>
       </c>
     </row>
@@ -5550,201 +5547,229 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t xml:space="preserve">Apr 2025</t>
-        </is>
+          <t xml:space="preserve">Jan-Mar 2025</t>
+        </is>
+      </c>
+      <c r="C17" s="11">
+        <v>5.71</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t xml:space="preserve">sampled farms: 16.7 % medium (5-10 %), 7.8 % high (10-15 %), 21.6 % very high (&gt; 15 %)</t>
+          <t xml:space="preserve">national average (13 of 15 departments hit; Santa Barbara 9.29 %, El Paraiso 7.91 %, Comayagua 7.20 %; worst varieties Obata and Catuai)</t>
         </is>
       </c>
       <c r="E17" s="17" t="inlineStr">
         <is>
-          <t xml:space="preserve">✔ USDA report (read)</t>
+          <t xml:space="preserve">✔ document read</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t xml:space="preserve">GAIN 2026</t>
+          <t xml:space="preserve">El Heraldo 13 May 2025 (read)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18">
+        <v>2025</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Apr 2025</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">sampled farms: 16.7 % medium (5-10 %), 7.8 % high (10-15 %), 21.6 % very high (&gt; 15 %)</t>
+        </is>
+      </c>
+      <c r="E18" s="17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">✔ USDA report (read)</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">GAIN 2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19">
         <v>2026</v>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="B19" t="inlineStr">
         <is>
           <t xml:space="preserve">end Jan 2026</t>
         </is>
       </c>
-      <c r="C18" s="11">
+      <c r="C19" s="11">
         <v>8.44</v>
       </c>
-      <c r="D18" t="inlineStr">
+      <c r="D19" t="inlineStr">
         <is>
           <t xml:space="preserve">national average incidence (from 7.57 %); departments 2.06-14.08 %; ~30 % of farms &gt; 10 %</t>
         </is>
       </c>
-      <c r="E18" s="17" t="inlineStr">
+      <c r="E19" s="17" t="inlineStr">
         <is>
           <t xml:space="preserve">✔ document read</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr">
+      <c r="F19" t="inlineStr">
         <is>
           <t xml:space="preserve">El Heraldo 15 Feb 2026 (read); GAIN 2026</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="3" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">IHCAFE rule of thumb</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="14" t="inlineStr">
-        <is>
-          <t xml:space="preserve">IHCAFE rule of thumb: rust damage of 15 % means about 20 % less production (GAIN 2017: "if the damage from rust reaches 15 percent, there could be a 20 percent reduction in production").</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="14" t="inlineStr">
         <is>
+          <t xml:space="preserve">IHCAFE rule of thumb: rust damage of 15 % means about 20 % less production (GAIN 2017: "if the damage from rust reaches 15 percent, there could be a 20 percent reduction in production").</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="14" t="inlineStr">
+        <is>
           <t xml:space="preserve">IHCAFE thresholds: 0-5 % low, 5-20 % medium (USDA 2022-2025).</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="4" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">Crop year</t>
         </is>
       </c>
-      <c r="B24" s="4" t="inlineStr">
+      <c r="B25" s="4" t="inlineStr">
         <is>
           <t xml:space="preserve">What USDA wrote that year (drought, disease, fertiliser, labour)</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2015/16</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t xml:space="preserve">El Nino drought: "Producers did not apply fertilizer due to the drought" (GAIN 2016).</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t xml:space="preserve">2016/17</t>
+          <t xml:space="preserve">2015/16</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t xml:space="preserve">First crop from plantings renewed after the 2012-14 rust (GAIN 2016).</t>
+          <t xml:space="preserve">El Nino drought: "Producers did not apply fertilizer due to the drought" (GAIN 2016).</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t xml:space="preserve">2017/18</t>
+          <t xml:space="preserve">2016/17</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t xml:space="preserve">Drought forecast; "Small farmers lack the resources to apply fertilizers" (GAIN 2017). Lempira hit by rust in 2016/17 (GAIN 2018).</t>
+          <t xml:space="preserve">First crop from plantings renewed after the 2012-14 rust (GAIN 2016).</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t xml:space="preserve">2019/20</t>
+          <t xml:space="preserve">2017/18</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t xml:space="preserve">Price 2.88 $/kg, lowest since 2007.</t>
+          <t xml:space="preserve">Drought forecast; "Small farmers lack the resources to apply fertilizers" (GAIN 2017). Lempira hit by rust in 2016/17 (GAIN 2018).</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t xml:space="preserve">2020/21</t>
+          <t xml:space="preserve">2019/20</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t xml:space="preserve">Bono Cafetalero: 25 188 t of fertiliser to 91 778 producers (GAIN 2021); hurricanes Eta and Iota in November.</t>
+          <t xml:space="preserve">Price 2.88 $/kg, lowest since 2007.</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t xml:space="preserve">2021/22</t>
+          <t xml:space="preserve">2020/21</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t xml:space="preserve">"cyclical decline in productivity after a widespread re-planting effort ten years ago" and rust (GAIN 2022); fertiliser prices up (Russia) (GAIN 2022).</t>
+          <t xml:space="preserve">Bono Cafetalero: 25 188 t of fertiliser to 91 778 producers (GAIN 2021); hurricanes Eta and Iota in November.</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t xml:space="preserve">2022/23</t>
+          <t xml:space="preserve">2021/22</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t xml:space="preserve">Less rust and "coffee drill bit" (berry borer) expected; high fertiliser costs (GAIN 2023).</t>
+          <t xml:space="preserve">"cyclical decline in productivity after a widespread re-planting effort ten years ago" and rust (GAIN 2022); fertiliser prices up (Russia) (GAIN 2022).</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t xml:space="preserve">2023/24</t>
+          <t xml:space="preserve">2022/23</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t xml:space="preserve">"high incidence of coffee rust and ongoing labor shortage" (GAIN 2024).</t>
+          <t xml:space="preserve">Less rust and "coffee drill bit" (berry borer) expected; high fertiliser costs (GAIN 2023).</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t xml:space="preserve">2024/25</t>
+          <t xml:space="preserve">2023/24</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t xml:space="preserve">Less rust, better labour availability, prices +81 % (GAIN 2025).</t>
+          <t xml:space="preserve">"high incidence of coffee rust and ongoing labor shortage" (GAIN 2024).</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
+          <t xml:space="preserve">2024/25</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Less rust, better labour availability, prices +81 % (GAIN 2025).</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
           <t xml:space="preserve">2025/26</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr">
+      <c r="B35" t="inlineStr">
         <is>
           <t xml:space="preserve">Parainema plantings harvested; rust up to 8.44 % by Jan 2026; fertiliser supply risk (Persian Gulf) (GAIN 2026).</t>
         </is>

</xml_diff>